<commit_message>
saisie d'ecran du fichier draw.io
</commit_message>
<xml_diff>
--- a/Diagramme de Gantt ECOTECH.xlsx
+++ b/Diagramme de Gantt ECOTECH.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{76A3087F-C11D-4D8F-8C20-47418E526455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA68A2F-E5AF-4DD7-83B6-4CAE3124144B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -173,9 +173,6 @@
     <t>Les entreprises trouveront également des modèles de facture, de feuille de temps, de suivi d’inventaire, d’états financiers et de planification de projet. Les enseignants et les étudiants pourront utiliser des ressources variées, notamment des emplois du temps, des carnets de notes et des feuilles de présence. Organisez votre vie famille avec des planificateurs de repas, des listes de contrôle et des journaux d’entraînement. Chaque modèle est minutieusement étudié, affiné et amélioré au fil du temps grâce aux commentaires de milliers d’utilisateurs.</t>
   </si>
   <si>
-    <t>pare feu</t>
-  </si>
-  <si>
     <t>Domaine ADDS</t>
   </si>
   <si>
@@ -295,6 +292,9 @@
 - Connexion via client de messagerie local
 - Validation d'envoie et de réception de mails entre 2 clients de messagerie sur serveur et client Windows
 </t>
+  </si>
+  <si>
+    <t>PARE FEU</t>
   </si>
 </sst>
 </file>
@@ -1430,41 +1430,41 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="168" fontId="27" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="27" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="27" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="27" fillId="0" borderId="3" xfId="9" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="8" applyFont="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="7" xfId="8" applyFont="1" applyBorder="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="9" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="10" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="9" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="8" applyFont="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="7" xfId="8" applyFont="1" applyBorder="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="27" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="27" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="27" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="27" fillId="0" borderId="3" xfId="9" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="54">
@@ -1867,10 +1867,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2157,7 +2153,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C1" s="27"/>
       <c r="D1" s="28"/>
@@ -2229,7 +2225,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="33" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -2299,16 +2295,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="36" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" s="85" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="83" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="86"/>
-      <c r="E3" s="90">
+      <c r="D3" s="84"/>
+      <c r="E3" s="82">
         <v>46035</v>
       </c>
-      <c r="F3" s="90"/>
+      <c r="F3" s="82"/>
       <c r="G3" s="31"/>
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
@@ -2373,96 +2369,96 @@
         <v>3</v>
       </c>
       <c r="B4" s="31"/>
-      <c r="C4" s="85" t="s">
+      <c r="C4" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="86"/>
+      <c r="D4" s="84"/>
       <c r="E4" s="37">
         <v>1</v>
       </c>
       <c r="F4" s="31"/>
       <c r="G4" s="31"/>
       <c r="H4" s="31"/>
-      <c r="I4" s="87">
+      <c r="I4" s="79">
         <f>I5</f>
         <v>46034</v>
       </c>
-      <c r="J4" s="88"/>
-      <c r="K4" s="88"/>
-      <c r="L4" s="88"/>
-      <c r="M4" s="88"/>
-      <c r="N4" s="88"/>
-      <c r="O4" s="89"/>
-      <c r="P4" s="87">
+      <c r="J4" s="80"/>
+      <c r="K4" s="80"/>
+      <c r="L4" s="80"/>
+      <c r="M4" s="80"/>
+      <c r="N4" s="80"/>
+      <c r="O4" s="81"/>
+      <c r="P4" s="79">
         <f>P5</f>
         <v>46041</v>
       </c>
-      <c r="Q4" s="88"/>
-      <c r="R4" s="88"/>
-      <c r="S4" s="88"/>
-      <c r="T4" s="88"/>
-      <c r="U4" s="88"/>
-      <c r="V4" s="89"/>
-      <c r="W4" s="87">
+      <c r="Q4" s="80"/>
+      <c r="R4" s="80"/>
+      <c r="S4" s="80"/>
+      <c r="T4" s="80"/>
+      <c r="U4" s="80"/>
+      <c r="V4" s="81"/>
+      <c r="W4" s="79">
         <f>W5</f>
         <v>46048</v>
       </c>
-      <c r="X4" s="88"/>
-      <c r="Y4" s="88"/>
-      <c r="Z4" s="88"/>
-      <c r="AA4" s="88"/>
-      <c r="AB4" s="88"/>
-      <c r="AC4" s="89"/>
-      <c r="AD4" s="87">
+      <c r="X4" s="80"/>
+      <c r="Y4" s="80"/>
+      <c r="Z4" s="80"/>
+      <c r="AA4" s="80"/>
+      <c r="AB4" s="80"/>
+      <c r="AC4" s="81"/>
+      <c r="AD4" s="79">
         <f>AD5</f>
         <v>46055</v>
       </c>
-      <c r="AE4" s="88"/>
-      <c r="AF4" s="88"/>
-      <c r="AG4" s="88"/>
-      <c r="AH4" s="88"/>
-      <c r="AI4" s="88"/>
-      <c r="AJ4" s="89"/>
-      <c r="AK4" s="87">
+      <c r="AE4" s="80"/>
+      <c r="AF4" s="80"/>
+      <c r="AG4" s="80"/>
+      <c r="AH4" s="80"/>
+      <c r="AI4" s="80"/>
+      <c r="AJ4" s="81"/>
+      <c r="AK4" s="79">
         <f>AK5</f>
         <v>46062</v>
       </c>
-      <c r="AL4" s="88"/>
-      <c r="AM4" s="88"/>
-      <c r="AN4" s="88"/>
-      <c r="AO4" s="88"/>
-      <c r="AP4" s="88"/>
-      <c r="AQ4" s="89"/>
-      <c r="AR4" s="87">
+      <c r="AL4" s="80"/>
+      <c r="AM4" s="80"/>
+      <c r="AN4" s="80"/>
+      <c r="AO4" s="80"/>
+      <c r="AP4" s="80"/>
+      <c r="AQ4" s="81"/>
+      <c r="AR4" s="79">
         <f>AR5</f>
         <v>46069</v>
       </c>
-      <c r="AS4" s="88"/>
-      <c r="AT4" s="88"/>
-      <c r="AU4" s="88"/>
-      <c r="AV4" s="88"/>
-      <c r="AW4" s="88"/>
-      <c r="AX4" s="89"/>
-      <c r="AY4" s="87">
+      <c r="AS4" s="80"/>
+      <c r="AT4" s="80"/>
+      <c r="AU4" s="80"/>
+      <c r="AV4" s="80"/>
+      <c r="AW4" s="80"/>
+      <c r="AX4" s="81"/>
+      <c r="AY4" s="79">
         <f>AY5</f>
         <v>46076</v>
       </c>
-      <c r="AZ4" s="88"/>
-      <c r="BA4" s="88"/>
-      <c r="BB4" s="88"/>
-      <c r="BC4" s="88"/>
-      <c r="BD4" s="88"/>
-      <c r="BE4" s="89"/>
-      <c r="BF4" s="87">
+      <c r="AZ4" s="80"/>
+      <c r="BA4" s="80"/>
+      <c r="BB4" s="80"/>
+      <c r="BC4" s="80"/>
+      <c r="BD4" s="80"/>
+      <c r="BE4" s="81"/>
+      <c r="BF4" s="79">
         <f>BF5</f>
         <v>46083</v>
       </c>
-      <c r="BG4" s="88"/>
-      <c r="BH4" s="88"/>
-      <c r="BI4" s="88"/>
-      <c r="BJ4" s="88"/>
-      <c r="BK4" s="88"/>
-      <c r="BL4" s="89"/>
+      <c r="BG4" s="80"/>
+      <c r="BH4" s="80"/>
+      <c r="BI4" s="80"/>
+      <c r="BJ4" s="80"/>
+      <c r="BK4" s="80"/>
+      <c r="BL4" s="81"/>
     </row>
     <row r="5" spans="1:64" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
@@ -3024,7 +3020,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="47" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C8" s="48"/>
       <c r="D8" s="49"/>
@@ -3098,13 +3094,13 @@
     </row>
     <row r="9" spans="1:64" s="2" customFormat="1" ht="111" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="15"/>
-      <c r="B9" s="82" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="82"/>
-      <c r="D9" s="82"/>
-      <c r="E9" s="82"/>
-      <c r="F9" s="82"/>
+      <c r="B9" s="85" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" s="85"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="85"/>
+      <c r="F9" s="85"/>
       <c r="G9" s="52"/>
       <c r="H9" s="52" t="str">
         <f t="shared" si="5"/>
@@ -3172,7 +3168,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="53" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C10" s="54"/>
       <c r="D10" s="55"/>
@@ -3246,13 +3242,13 @@
     </row>
     <row r="11" spans="1:64" s="2" customFormat="1" ht="85.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14"/>
-      <c r="B11" s="80" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="80"/>
-      <c r="D11" s="80"/>
-      <c r="E11" s="80"/>
-      <c r="F11" s="80"/>
+      <c r="B11" s="88" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="88"/>
+      <c r="D11" s="88"/>
+      <c r="E11" s="88"/>
+      <c r="F11" s="88"/>
       <c r="G11" s="52"/>
       <c r="H11" s="52" t="str">
         <f t="shared" si="5"/>
@@ -3317,13 +3313,13 @@
     </row>
     <row r="12" spans="1:64" s="2" customFormat="1" ht="98.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14"/>
-      <c r="B12" s="80" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="80"/>
-      <c r="D12" s="80"/>
-      <c r="E12" s="80"/>
-      <c r="F12" s="80"/>
+      <c r="B12" s="88" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="88"/>
+      <c r="D12" s="88"/>
+      <c r="E12" s="88"/>
+      <c r="F12" s="88"/>
       <c r="G12" s="52"/>
       <c r="H12" s="52" t="str">
         <f t="shared" si="5"/>
@@ -3388,13 +3384,13 @@
     </row>
     <row r="13" spans="1:64" s="2" customFormat="1" ht="99" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14"/>
-      <c r="B13" s="80" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="80"/>
-      <c r="D13" s="80"/>
-      <c r="E13" s="80"/>
-      <c r="F13" s="80"/>
+      <c r="B13" s="88" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="88"/>
+      <c r="D13" s="88"/>
+      <c r="E13" s="88"/>
+      <c r="F13" s="88"/>
       <c r="G13" s="52"/>
       <c r="H13" s="52" t="str">
         <f t="shared" si="5"/>
@@ -3461,13 +3457,13 @@
       <c r="A14" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="80" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="80"/>
-      <c r="D14" s="80"/>
-      <c r="E14" s="80"/>
-      <c r="F14" s="80"/>
+      <c r="B14" s="88" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="88"/>
+      <c r="D14" s="88"/>
+      <c r="E14" s="88"/>
+      <c r="F14" s="88"/>
       <c r="G14" s="52"/>
       <c r="H14" s="52" t="str">
         <f t="shared" si="5"/>
@@ -3533,7 +3529,7 @@
     <row r="15" spans="1:64" s="2" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14"/>
       <c r="B15" s="59" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C15" s="60"/>
       <c r="D15" s="61"/>
@@ -3570,7 +3566,7 @@
       <c r="AB15" s="63"/>
       <c r="AC15" s="63"/>
       <c r="AD15" s="63" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AE15" s="63"/>
       <c r="AF15" s="46"/>
@@ -3609,13 +3605,13 @@
     </row>
     <row r="16" spans="1:64" s="2" customFormat="1" ht="123" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="14"/>
-      <c r="B16" s="81" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" s="81"/>
-      <c r="D16" s="81"/>
-      <c r="E16" s="81"/>
-      <c r="F16" s="81"/>
+      <c r="B16" s="90" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="90"/>
+      <c r="D16" s="90"/>
+      <c r="E16" s="90"/>
+      <c r="F16" s="90"/>
       <c r="G16" s="52"/>
       <c r="H16" s="52" t="str">
         <f t="shared" si="5"/>
@@ -3681,7 +3677,7 @@
     <row r="17" spans="1:88" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14"/>
       <c r="B17" s="65" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C17" s="66"/>
       <c r="D17" s="67"/>
@@ -3755,11 +3751,11 @@
     </row>
     <row r="18" spans="1:88" s="2" customFormat="1" ht="98.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14"/>
-      <c r="B18" s="83" t="s">
-        <v>51</v>
-      </c>
-      <c r="C18" s="83"/>
-      <c r="D18" s="83"/>
+      <c r="B18" s="86" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="86"/>
+      <c r="D18" s="86"/>
       <c r="E18" s="68"/>
       <c r="F18" s="68"/>
       <c r="G18" s="52"/>
@@ -3827,7 +3823,7 @@
     <row r="19" spans="1:88" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="14"/>
       <c r="B19" s="47" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C19" s="48"/>
       <c r="D19" s="49"/>
@@ -3903,11 +3899,11 @@
     </row>
     <row r="20" spans="1:88" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14"/>
-      <c r="B20" s="84" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" s="84"/>
-      <c r="D20" s="84"/>
+      <c r="B20" s="87" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="87"/>
+      <c r="D20" s="87"/>
       <c r="E20" s="69"/>
       <c r="F20" s="69"/>
       <c r="G20" s="52"/>
@@ -3976,11 +3972,11 @@
     </row>
     <row r="21" spans="1:88" s="2" customFormat="1" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="14"/>
-      <c r="B21" s="84" t="s">
-        <v>53</v>
-      </c>
-      <c r="C21" s="84"/>
-      <c r="D21" s="84"/>
+      <c r="B21" s="87" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="87"/>
+      <c r="D21" s="87"/>
       <c r="E21" s="69"/>
       <c r="F21" s="69"/>
       <c r="G21" s="52"/>
@@ -4052,7 +4048,7 @@
         <v>8</v>
       </c>
       <c r="B22" s="53" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C22" s="54"/>
       <c r="D22" s="55"/>
@@ -4128,11 +4124,11 @@
     </row>
     <row r="23" spans="1:88" s="23" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="22"/>
-      <c r="B23" s="80" t="s">
-        <v>54</v>
-      </c>
-      <c r="C23" s="80"/>
-      <c r="D23" s="80"/>
+      <c r="B23" s="88" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="88"/>
+      <c r="D23" s="88"/>
       <c r="E23" s="70"/>
       <c r="F23" s="70"/>
       <c r="G23" s="71"/>
@@ -4201,11 +4197,11 @@
     </row>
     <row r="24" spans="1:88" s="23" customFormat="1" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="22"/>
-      <c r="B24" s="80" t="s">
-        <v>55</v>
-      </c>
-      <c r="C24" s="80"/>
-      <c r="D24" s="80"/>
+      <c r="B24" s="88" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="88"/>
+      <c r="D24" s="88"/>
       <c r="E24" s="70"/>
       <c r="F24" s="70"/>
       <c r="G24" s="71"/>
@@ -4275,7 +4271,7 @@
     <row r="25" spans="1:88" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14"/>
       <c r="B25" s="59" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C25" s="60"/>
       <c r="D25" s="61"/>
@@ -4347,18 +4343,18 @@
       <c r="BK25" s="46"/>
       <c r="BL25" s="46"/>
       <c r="BR25" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="BU25" s="17"/>
       <c r="CJ25" s="18"/>
     </row>
     <row r="26" spans="1:88" s="2" customFormat="1" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="14"/>
-      <c r="B26" s="81" t="s">
-        <v>57</v>
-      </c>
-      <c r="C26" s="81"/>
-      <c r="D26" s="81"/>
+      <c r="B26" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="90"/>
+      <c r="D26" s="90"/>
       <c r="E26" s="74"/>
       <c r="F26" s="74"/>
       <c r="G26" s="52"/>
@@ -4427,11 +4423,11 @@
     </row>
     <row r="27" spans="1:88" s="2" customFormat="1" ht="109.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="14"/>
-      <c r="B27" s="81" t="s">
-        <v>58</v>
-      </c>
-      <c r="C27" s="81"/>
-      <c r="D27" s="81"/>
+      <c r="B27" s="90" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" s="90"/>
+      <c r="D27" s="90"/>
       <c r="E27" s="74"/>
       <c r="F27" s="74"/>
       <c r="G27" s="52"/>
@@ -4501,7 +4497,7 @@
     <row r="28" spans="1:88" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="14"/>
       <c r="B28" s="65" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C28" s="66"/>
       <c r="D28" s="67"/>
@@ -4591,11 +4587,11 @@
     </row>
     <row r="29" spans="1:88" s="2" customFormat="1" ht="90" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="14"/>
-      <c r="B29" s="79" t="s">
-        <v>59</v>
-      </c>
-      <c r="C29" s="79"/>
-      <c r="D29" s="79"/>
+      <c r="B29" s="89" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="89"/>
+      <c r="D29" s="89"/>
       <c r="E29" s="68"/>
       <c r="F29" s="68"/>
       <c r="G29" s="52"/>
@@ -4664,11 +4660,11 @@
     </row>
     <row r="30" spans="1:88" s="2" customFormat="1" ht="116.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="14"/>
-      <c r="B30" s="79" t="s">
-        <v>60</v>
-      </c>
-      <c r="C30" s="79"/>
-      <c r="D30" s="79"/>
+      <c r="B30" s="89" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" s="89"/>
+      <c r="D30" s="89"/>
       <c r="E30" s="68"/>
       <c r="F30" s="68"/>
       <c r="G30" s="52"/>
@@ -5029,17 +5025,13 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="BF4:BL4"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="I4:O4"/>
-    <mergeCell ref="P4:V4"/>
-    <mergeCell ref="W4:AC4"/>
-    <mergeCell ref="AD4:AJ4"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="AK4:AQ4"/>
-    <mergeCell ref="AR4:AX4"/>
-    <mergeCell ref="AY4:BE4"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="B20:D20"/>
@@ -5048,13 +5040,17 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="AK4:AQ4"/>
+    <mergeCell ref="AR4:AX4"/>
+    <mergeCell ref="AY4:BE4"/>
+    <mergeCell ref="BF4:BL4"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="I4:O4"/>
+    <mergeCell ref="P4:V4"/>
+    <mergeCell ref="W4:AC4"/>
+    <mergeCell ref="AD4:AJ4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D8 D10 D15 D17 D19 D22 D25 D28">
     <cfRule type="dataBar" priority="14">
@@ -5247,23 +5243,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5555,22 +5540,29 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5597,9 +5589,13 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>